<commit_message>
Mating connector part added
</commit_message>
<xml_diff>
--- a/(Updated) BOM_SB_BIU_S2 v2.2_Changes.xlsx
+++ b/(Updated) BOM_SB_BIU_S2 v2.2_Changes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\robertMeares-VCU-BCU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA68FFA2-7790-4B9D-942C-3DAC75DE6286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B725AB-1A25-41B7-9AF0-FD1C5F9F7E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="172">
   <si>
     <t xml:space="preserve">Index  Revised: </t>
   </si>
@@ -547,6 +547,12 @@
   </si>
   <si>
     <t>RC0603FR-071K2L</t>
+  </si>
+  <si>
+    <t>T2M-110-01-L-D-RA-WT</t>
+  </si>
+  <si>
+    <t>Suggested Connector</t>
   </si>
 </sst>
 </file>
@@ -841,21 +847,6 @@
   </cellStyleXfs>
   <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -964,6 +955,21 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1484,1779 +1490,1783 @@
   <dimension ref="A1:AML57"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="6"/>
-    <col min="3" max="3" width="36.5703125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="42.85546875" style="6" customWidth="1"/>
-    <col min="6" max="8" width="22.7109375" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
-    <col min="10" max="13" width="11.5703125" style="6" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" style="6" customWidth="1"/>
-    <col min="15" max="16" width="11.5703125" style="6" customWidth="1"/>
-    <col min="17" max="17" width="20.85546875" style="6" customWidth="1"/>
-    <col min="18" max="20" width="11.5703125" style="6" customWidth="1"/>
-    <col min="21" max="1026" width="9.140625" style="6"/>
+    <col min="1" max="1" width="17.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="36.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="1" customWidth="1"/>
+    <col min="5" max="5" width="42.85546875" style="1" customWidth="1"/>
+    <col min="6" max="8" width="22.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.140625" style="1" customWidth="1"/>
+    <col min="10" max="13" width="11.5703125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" style="1" customWidth="1"/>
+    <col min="15" max="16" width="11.5703125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="20.85546875" style="1" customWidth="1"/>
+    <col min="18" max="20" width="11.5703125" style="1" customWidth="1"/>
+    <col min="21" max="1026" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5">
+      <c r="B1" s="39">
         <v>44883</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="40">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
     </row>
     <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
     </row>
     <row r="6" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
     </row>
     <row r="10" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9" t="s">
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="K10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="L10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="M10" s="9" t="s">
+      <c r="M10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O10" s="12" t="s">
+      <c r="O10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P10" s="12" t="s">
+      <c r="P10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q10" s="12" t="s">
+      <c r="Q10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="R10" s="13" t="s">
+      <c r="R10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="S10" s="13" t="s">
+      <c r="S10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="T10" s="13" t="s">
+      <c r="T10" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
+      <c r="A11" s="9">
         <v>1</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="9">
         <v>17</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="16" t="s">
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="17">
+      <c r="J11" s="12">
         <v>402</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M11" s="16">
+      <c r="M11" s="11">
         <v>19</v>
       </c>
-      <c r="N11" s="18" t="s">
+      <c r="N11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="O11" s="19">
+      <c r="O11" s="14">
         <v>0.1</v>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="14">
         <f>B11*O11</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="Q11" s="19">
+      <c r="Q11" s="14">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="R11" s="19">
+      <c r="R11" s="14">
         <f>B11*Q11</f>
         <v>0.153</v>
       </c>
-      <c r="S11" s="19">
+      <c r="S11" s="14">
         <f>0.4*Q11</f>
         <v>3.5999999999999999E-3</v>
       </c>
-      <c r="T11" s="19">
+      <c r="T11" s="14">
         <f>B11*S11</f>
         <v>6.1199999999999997E-2</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="14">
+      <c r="A12" s="9">
         <v>2</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="9">
         <v>1</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="20" t="s">
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="16">
         <v>603</v>
       </c>
-      <c r="K12" s="16" t="s">
+      <c r="K12" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L12" s="20" t="s">
+      <c r="L12" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="20">
+      <c r="M12" s="15">
         <v>28</v>
       </c>
-      <c r="N12" s="22"/>
-      <c r="O12" s="19">
+      <c r="N12" s="17"/>
+      <c r="O12" s="14">
         <v>0.7</v>
       </c>
-      <c r="P12" s="19">
+      <c r="P12" s="14">
         <f>B12*O12</f>
         <v>0.7</v>
       </c>
-      <c r="Q12" s="19">
+      <c r="Q12" s="14">
         <v>0.2</v>
       </c>
-      <c r="R12" s="19">
+      <c r="R12" s="14">
         <f>B12*Q12</f>
         <v>0.2</v>
       </c>
-      <c r="S12" s="19">
+      <c r="S12" s="14">
         <f>0.4*Q12</f>
         <v>8.0000000000000016E-2</v>
       </c>
-      <c r="T12" s="19">
+      <c r="T12" s="14">
         <f>B12*S12</f>
         <v>8.0000000000000016E-2</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
+      <c r="A13" s="9">
         <v>3</v>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="9">
         <v>5</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="20" t="s">
+      <c r="G13" s="35"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="16">
         <v>603</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L13" s="20" t="s">
+      <c r="L13" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="20">
+      <c r="M13" s="15">
         <v>14</v>
       </c>
-      <c r="N13" s="22"/>
-      <c r="O13" s="19">
+      <c r="N13" s="17"/>
+      <c r="O13" s="14">
         <v>0.17</v>
       </c>
-      <c r="P13" s="19">
+      <c r="P13" s="14">
         <f>B13*O13</f>
         <v>0.85000000000000009</v>
       </c>
-      <c r="Q13" s="19">
+      <c r="Q13" s="14">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="R13" s="19">
+      <c r="R13" s="14">
         <f>B13*Q13</f>
         <v>0.185</v>
       </c>
-      <c r="S13" s="19">
+      <c r="S13" s="14">
         <f>0.4*Q13</f>
         <v>1.4800000000000001E-2</v>
       </c>
-      <c r="T13" s="19">
+      <c r="T13" s="14">
         <f>B13*S13</f>
         <v>7.400000000000001E-2</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
+      <c r="A14" s="9">
         <v>4</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="9">
         <v>6</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="20" t="s">
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="16">
         <v>603</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L14" s="20" t="s">
+      <c r="L14" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="20">
+      <c r="M14" s="15">
         <v>31</v>
       </c>
-      <c r="N14" s="22"/>
-      <c r="O14" s="19">
+      <c r="N14" s="17"/>
+      <c r="O14" s="14">
         <v>0.28000000000000003</v>
       </c>
-      <c r="P14" s="19">
+      <c r="P14" s="14">
         <f>B14*O14</f>
         <v>1.6800000000000002</v>
       </c>
-      <c r="Q14" s="19">
+      <c r="Q14" s="14">
         <v>0.06</v>
       </c>
-      <c r="R14" s="19">
+      <c r="R14" s="14">
         <f>B14*Q14</f>
         <v>0.36</v>
       </c>
-      <c r="S14" s="19">
+      <c r="S14" s="14">
         <f>0.4*Q14</f>
         <v>2.4E-2</v>
       </c>
-      <c r="T14" s="19">
+      <c r="T14" s="14">
         <f>B14*S14</f>
         <v>0.14400000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14">
+      <c r="A15" s="9">
         <v>5</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="9">
         <v>3</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="20" t="s">
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="J15" s="21">
+      <c r="J15" s="16">
         <v>1206</v>
       </c>
-      <c r="K15" s="16" t="s">
+      <c r="K15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L15" s="20" t="s">
+      <c r="L15" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="20">
+      <c r="M15" s="15">
         <v>28</v>
       </c>
-      <c r="N15" s="22" t="s">
+      <c r="N15" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="O15" s="19"/>
-      <c r="P15" s="19"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="19"/>
-      <c r="S15" s="19"/>
-      <c r="T15" s="19"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
     </row>
     <row r="16" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="14">
+      <c r="A16" s="9">
         <v>6</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="9">
         <v>4</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="23" t="s">
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="J16" s="21" t="s">
+      <c r="J16" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K16" s="20" t="s">
+      <c r="K16" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="L16" s="20" t="s">
+      <c r="L16" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M16" s="20">
+      <c r="M16" s="15">
         <v>15</v>
       </c>
-      <c r="N16" s="24" t="s">
+      <c r="N16" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="O16" s="19">
+      <c r="O16" s="14">
         <v>0.37</v>
       </c>
-      <c r="P16" s="19">
+      <c r="P16" s="14">
         <f t="shared" ref="P16:P35" si="0">B16*O16</f>
         <v>1.48</v>
       </c>
-      <c r="Q16" s="19">
+      <c r="Q16" s="14">
         <v>0.09</v>
       </c>
-      <c r="R16" s="19">
+      <c r="R16" s="14">
         <f t="shared" ref="R16:R34" si="1">B16*Q16</f>
         <v>0.36</v>
       </c>
-      <c r="S16" s="19">
+      <c r="S16" s="14">
         <f t="shared" ref="S16:S34" si="2">0.4*Q16</f>
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="T16" s="19">
+      <c r="T16" s="14">
         <f t="shared" ref="T16:T35" si="3">B16*S16</f>
         <v>0.14399999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14">
+      <c r="A17" s="9">
         <v>7</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="9">
         <v>1</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E17" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="40"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="20" t="s">
+      <c r="G17" s="35" t="s">
+        <v>170</v>
+      </c>
+      <c r="H17" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I17" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="J17" s="21" t="s">
+      <c r="J17" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K17" s="20" t="s">
+      <c r="K17" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="L17" s="20" t="s">
+      <c r="L17" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="M17" s="20">
+      <c r="M17" s="15">
         <v>12</v>
       </c>
-      <c r="N17" s="22"/>
-      <c r="O17" s="19">
+      <c r="N17" s="17"/>
+      <c r="O17" s="14">
         <v>2.7</v>
       </c>
-      <c r="P17" s="19">
+      <c r="P17" s="14">
         <f t="shared" si="0"/>
         <v>2.7</v>
       </c>
-      <c r="Q17" s="19">
+      <c r="Q17" s="14">
         <v>1.45</v>
       </c>
-      <c r="R17" s="19">
+      <c r="R17" s="14">
         <f t="shared" si="1"/>
         <v>1.45</v>
       </c>
-      <c r="S17" s="19">
+      <c r="S17" s="14">
         <f t="shared" si="2"/>
         <v>0.57999999999999996</v>
       </c>
-      <c r="T17" s="19">
+      <c r="T17" s="14">
         <f t="shared" si="3"/>
         <v>0.57999999999999996</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="14">
+      <c r="A18" s="9">
         <v>8</v>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="9">
         <v>1</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="20" t="s">
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="21"/>
-      <c r="K18" s="20" t="s">
+      <c r="J18" s="16"/>
+      <c r="K18" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="L18" s="20" t="s">
+      <c r="L18" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M18" s="20">
+      <c r="M18" s="15">
         <v>17</v>
       </c>
-      <c r="N18" s="22"/>
-      <c r="O18" s="19">
+      <c r="N18" s="17"/>
+      <c r="O18" s="14">
         <v>8.23</v>
       </c>
-      <c r="P18" s="19">
+      <c r="P18" s="14">
         <f t="shared" si="0"/>
         <v>8.23</v>
       </c>
-      <c r="Q18" s="19">
+      <c r="Q18" s="14">
         <v>4.9000000000000004</v>
       </c>
-      <c r="R18" s="19">
+      <c r="R18" s="14">
         <f t="shared" si="1"/>
         <v>4.9000000000000004</v>
       </c>
-      <c r="S18" s="19">
+      <c r="S18" s="14">
         <f t="shared" si="2"/>
         <v>1.9600000000000002</v>
       </c>
-      <c r="T18" s="19">
+      <c r="T18" s="14">
         <f t="shared" si="3"/>
         <v>1.9600000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="14">
+      <c r="A19" s="9">
         <v>9</v>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="9">
         <v>2</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="20" t="s">
+      <c r="G19" s="35"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="J19" s="21">
+      <c r="J19" s="16">
         <v>805</v>
       </c>
-      <c r="K19" s="20" t="s">
+      <c r="K19" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="L19" s="20" t="s">
+      <c r="L19" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M19" s="20">
+      <c r="M19" s="15">
         <v>19</v>
       </c>
-      <c r="N19" s="22"/>
-      <c r="O19" s="19">
+      <c r="N19" s="17"/>
+      <c r="O19" s="14">
         <v>0.28999999999999998</v>
       </c>
-      <c r="P19" s="19">
+      <c r="P19" s="14">
         <f t="shared" si="0"/>
         <v>0.57999999999999996</v>
       </c>
-      <c r="Q19" s="19">
+      <c r="Q19" s="14">
         <v>0.09</v>
       </c>
-      <c r="R19" s="19">
+      <c r="R19" s="14">
         <f t="shared" si="1"/>
         <v>0.18</v>
       </c>
-      <c r="S19" s="19">
+      <c r="S19" s="14">
         <f t="shared" si="2"/>
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="T19" s="19">
+      <c r="T19" s="14">
         <f t="shared" si="3"/>
         <v>7.1999999999999995E-2</v>
       </c>
     </row>
     <row r="20" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
+      <c r="A20" s="9">
         <v>10</v>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="9">
         <v>4</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="20" t="s">
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="J20" s="21">
+      <c r="J20" s="16">
         <v>805</v>
       </c>
-      <c r="K20" s="20" t="s">
+      <c r="K20" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="L20" s="20" t="s">
+      <c r="L20" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="20">
+      <c r="M20" s="15">
         <v>10</v>
       </c>
-      <c r="N20" s="22" t="s">
+      <c r="N20" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="O20" s="19">
+      <c r="O20" s="14">
         <v>0.11</v>
       </c>
-      <c r="P20" s="19">
+      <c r="P20" s="14">
         <f t="shared" si="0"/>
         <v>0.44</v>
       </c>
-      <c r="Q20" s="19">
+      <c r="Q20" s="14">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="R20" s="19">
+      <c r="R20" s="14">
         <f t="shared" si="1"/>
         <v>0.11600000000000001</v>
       </c>
-      <c r="S20" s="19">
+      <c r="S20" s="14">
         <f t="shared" si="2"/>
         <v>1.1600000000000001E-2</v>
       </c>
-      <c r="T20" s="19">
+      <c r="T20" s="14">
         <f t="shared" si="3"/>
         <v>4.6400000000000004E-2</v>
       </c>
     </row>
     <row r="21" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="14">
+      <c r="A21" s="9">
         <v>11</v>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="9">
         <v>5</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="20" t="s">
+      <c r="G21" s="35"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="J21" s="21">
+      <c r="J21" s="16">
         <v>805</v>
       </c>
-      <c r="K21" s="20" t="s">
+      <c r="K21" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="L21" s="20" t="s">
+      <c r="L21" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M21" s="20">
+      <c r="M21" s="15">
         <v>8</v>
       </c>
-      <c r="N21" s="22"/>
-      <c r="O21" s="19">
+      <c r="N21" s="17"/>
+      <c r="O21" s="14">
         <v>0.14000000000000001</v>
       </c>
-      <c r="P21" s="19">
+      <c r="P21" s="14">
         <f t="shared" si="0"/>
         <v>0.70000000000000007</v>
       </c>
-      <c r="Q21" s="19">
+      <c r="Q21" s="14">
         <v>0.04</v>
       </c>
-      <c r="R21" s="19">
+      <c r="R21" s="14">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="S21" s="19">
+      <c r="S21" s="14">
         <f t="shared" si="2"/>
         <v>1.6E-2</v>
       </c>
-      <c r="T21" s="19">
+      <c r="T21" s="14">
         <f t="shared" si="3"/>
         <v>0.08</v>
       </c>
     </row>
     <row r="22" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
+      <c r="A22" s="9">
         <v>12</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="9">
         <v>2</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="20" t="s">
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="J22" s="21" t="s">
+      <c r="J22" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="K22" s="20" t="s">
+      <c r="K22" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="L22" s="20" t="s">
+      <c r="L22" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M22" s="20">
+      <c r="M22" s="15">
         <v>7</v>
       </c>
-      <c r="N22" s="22"/>
-      <c r="O22" s="19">
+      <c r="N22" s="17"/>
+      <c r="O22" s="14">
         <v>2.9</v>
       </c>
-      <c r="P22" s="19">
+      <c r="P22" s="14">
         <f t="shared" si="0"/>
         <v>5.8</v>
       </c>
-      <c r="Q22" s="19">
+      <c r="Q22" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="R22" s="19">
+      <c r="R22" s="14">
         <f t="shared" si="1"/>
         <v>2.2000000000000002</v>
       </c>
-      <c r="S22" s="19">
+      <c r="S22" s="14">
         <f t="shared" si="2"/>
         <v>0.44000000000000006</v>
       </c>
-      <c r="T22" s="19">
+      <c r="T22" s="14">
         <f t="shared" si="3"/>
         <v>0.88000000000000012</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="14">
+      <c r="A23" s="9">
         <v>13</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="9">
         <v>13</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="20" t="s">
+      <c r="G23" s="35"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="J23" s="21">
+      <c r="J23" s="16">
         <v>603</v>
       </c>
-      <c r="K23" s="20" t="s">
+      <c r="K23" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L23" s="20" t="s">
+      <c r="L23" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M23" s="20">
+      <c r="M23" s="15">
         <v>14</v>
       </c>
-      <c r="N23" s="22" t="s">
+      <c r="N23" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="14">
         <v>0.1</v>
       </c>
-      <c r="P23" s="19">
+      <c r="P23" s="14">
         <f t="shared" si="0"/>
         <v>1.3</v>
       </c>
-      <c r="Q23" s="19">
+      <c r="Q23" s="14">
         <v>0.01</v>
       </c>
-      <c r="R23" s="19">
+      <c r="R23" s="14">
         <f t="shared" si="1"/>
         <v>0.13</v>
       </c>
-      <c r="S23" s="19">
+      <c r="S23" s="14">
         <f t="shared" si="2"/>
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="T23" s="19">
+      <c r="T23" s="14">
         <f t="shared" si="3"/>
         <v>5.2000000000000005E-2</v>
       </c>
     </row>
     <row r="24" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
+      <c r="A24" s="9">
         <v>14</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="9">
         <v>2</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="D24" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="G24" s="40"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="20" t="s">
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="J24" s="21">
+      <c r="J24" s="16">
         <v>603</v>
       </c>
-      <c r="K24" s="20" t="s">
+      <c r="K24" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L24" s="20" t="s">
+      <c r="L24" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M24" s="20">
+      <c r="M24" s="15">
         <v>24</v>
       </c>
-      <c r="N24" s="22"/>
-      <c r="O24" s="19">
+      <c r="N24" s="17"/>
+      <c r="O24" s="14">
         <v>0.1</v>
       </c>
-      <c r="P24" s="19">
+      <c r="P24" s="14">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="Q24" s="19">
+      <c r="Q24" s="14">
         <v>0.04</v>
       </c>
-      <c r="R24" s="19">
+      <c r="R24" s="14">
         <f t="shared" si="1"/>
         <v>0.08</v>
       </c>
-      <c r="S24" s="19">
+      <c r="S24" s="14">
         <f t="shared" si="2"/>
         <v>1.6E-2</v>
       </c>
-      <c r="T24" s="19">
+      <c r="T24" s="14">
         <f t="shared" si="3"/>
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
     <row r="25" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="14">
+      <c r="A25" s="9">
         <v>15</v>
       </c>
-      <c r="B25" s="14">
+      <c r="B25" s="9">
         <v>4</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="20" t="s">
+      <c r="G25" s="35"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="J25" s="21">
+      <c r="J25" s="16">
         <v>402</v>
       </c>
-      <c r="K25" s="20" t="s">
+      <c r="K25" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L25" s="20" t="s">
+      <c r="L25" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M25" s="20">
+      <c r="M25" s="15">
         <v>35</v>
       </c>
-      <c r="N25" s="22"/>
-      <c r="O25" s="19">
+      <c r="N25" s="17"/>
+      <c r="O25" s="14">
         <v>0.1</v>
       </c>
-      <c r="P25" s="19">
+      <c r="P25" s="14">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="Q25" s="19">
+      <c r="Q25" s="14">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="R25" s="19">
+      <c r="R25" s="14">
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="S25" s="19">
+      <c r="S25" s="14">
         <f t="shared" si="2"/>
         <v>2E-3</v>
       </c>
-      <c r="T25" s="19">
+      <c r="T25" s="14">
         <f t="shared" si="3"/>
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="26" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
+      <c r="A26" s="9">
         <v>16</v>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="9">
         <v>4</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="G26" s="40"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="20" t="s">
+      <c r="G26" s="35"/>
+      <c r="H26" s="35"/>
+      <c r="I26" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="J26" s="21">
+      <c r="J26" s="16">
         <v>603</v>
       </c>
-      <c r="K26" s="20" t="s">
+      <c r="K26" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L26" s="20" t="s">
+      <c r="L26" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M26" s="20">
+      <c r="M26" s="15">
         <v>29</v>
       </c>
-      <c r="N26" s="22" t="s">
+      <c r="N26" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="O26" s="19">
+      <c r="O26" s="14">
         <v>0.1</v>
       </c>
-      <c r="P26" s="19">
+      <c r="P26" s="14">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="Q26" s="19">
+      <c r="Q26" s="14">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="R26" s="19">
+      <c r="R26" s="14">
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="S26" s="19">
+      <c r="S26" s="14">
         <f t="shared" si="2"/>
         <v>2E-3</v>
       </c>
-      <c r="T26" s="19">
+      <c r="T26" s="14">
         <f t="shared" si="3"/>
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="14">
+      <c r="A27" s="9">
         <v>17</v>
       </c>
-      <c r="B27" s="14">
+      <c r="B27" s="9">
         <v>2</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D27" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="20" t="s">
+      <c r="G27" s="35"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="J27" s="21">
+      <c r="J27" s="16">
         <v>603</v>
       </c>
-      <c r="K27" s="20" t="s">
+      <c r="K27" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L27" s="20" t="s">
+      <c r="L27" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M27" s="20">
+      <c r="M27" s="15">
         <v>24</v>
       </c>
-      <c r="N27" s="22" t="s">
+      <c r="N27" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="O27" s="19">
+      <c r="O27" s="14">
         <v>0.1</v>
       </c>
-      <c r="P27" s="19">
+      <c r="P27" s="14">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="Q27" s="19">
+      <c r="Q27" s="14">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="R27" s="19">
+      <c r="R27" s="14">
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="S27" s="19">
+      <c r="S27" s="14">
         <f t="shared" si="2"/>
         <v>2E-3</v>
       </c>
-      <c r="T27" s="19">
+      <c r="T27" s="14">
         <f t="shared" si="3"/>
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
     <row r="28" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="14">
+      <c r="A28" s="9">
         <v>18</v>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="9">
         <v>1</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="20" t="s">
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="J28" s="21" t="s">
+      <c r="J28" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="K28" s="20" t="s">
+      <c r="K28" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L28" s="20" t="s">
+      <c r="L28" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M28" s="20">
+      <c r="M28" s="15">
         <v>16</v>
       </c>
-      <c r="N28" s="22"/>
-      <c r="O28" s="19">
+      <c r="N28" s="17"/>
+      <c r="O28" s="14">
         <v>2.46</v>
       </c>
-      <c r="P28" s="19">
+      <c r="P28" s="14">
         <f t="shared" si="0"/>
         <v>2.46</v>
       </c>
-      <c r="Q28" s="19">
+      <c r="Q28" s="14">
         <v>1.1299999999999999</v>
       </c>
-      <c r="R28" s="19">
+      <c r="R28" s="14">
         <f t="shared" si="1"/>
         <v>1.1299999999999999</v>
       </c>
-      <c r="S28" s="19">
+      <c r="S28" s="14">
         <f t="shared" si="2"/>
         <v>0.45199999999999996</v>
       </c>
-      <c r="T28" s="19">
+      <c r="T28" s="14">
         <f t="shared" si="3"/>
         <v>0.45199999999999996</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="14">
+      <c r="A29" s="9">
         <v>19</v>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="9">
         <v>1</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="E29" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="F29" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="20" t="s">
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="J29" s="21" t="s">
+      <c r="J29" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="K29" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="L29" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M29" s="20">
+      <c r="M29" s="15">
         <v>6</v>
       </c>
-      <c r="N29" s="22"/>
-      <c r="O29" s="19">
+      <c r="N29" s="17"/>
+      <c r="O29" s="14">
         <v>1.6</v>
       </c>
-      <c r="P29" s="19">
+      <c r="P29" s="14">
         <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
-      <c r="Q29" s="19">
+      <c r="Q29" s="14">
         <v>0.6</v>
       </c>
-      <c r="R29" s="19">
+      <c r="R29" s="14">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="S29" s="19">
+      <c r="S29" s="14">
         <f t="shared" si="2"/>
         <v>0.24</v>
       </c>
-      <c r="T29" s="19">
+      <c r="T29" s="14">
         <f t="shared" si="3"/>
         <v>0.24</v>
       </c>
     </row>
     <row r="30" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="14">
+      <c r="A30" s="9">
         <v>20</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="9">
         <v>1</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C30" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="F30" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="20" t="s">
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="J30" s="21" t="s">
+      <c r="J30" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="K30" s="20" t="s">
+      <c r="K30" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L30" s="20" t="s">
+      <c r="L30" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M30" s="20">
+      <c r="M30" s="15">
         <v>6</v>
       </c>
-      <c r="N30" s="22"/>
-      <c r="O30" s="19">
+      <c r="N30" s="17"/>
+      <c r="O30" s="14">
         <v>0.63</v>
       </c>
-      <c r="P30" s="19">
+      <c r="P30" s="14">
         <f t="shared" si="0"/>
         <v>0.63</v>
       </c>
-      <c r="Q30" s="19">
+      <c r="Q30" s="14">
         <v>0.2</v>
       </c>
-      <c r="R30" s="19">
+      <c r="R30" s="14">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="S30" s="19">
+      <c r="S30" s="14">
         <f t="shared" si="2"/>
         <v>8.0000000000000016E-2</v>
       </c>
-      <c r="T30" s="19">
+      <c r="T30" s="14">
         <f t="shared" si="3"/>
         <v>8.0000000000000016E-2</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="14">
+      <c r="A31" s="9">
         <v>21</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="9">
         <v>1</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="C31" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="F31" s="14" t="s">
+      <c r="F31" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="20" t="s">
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="J31" s="21" t="s">
+      <c r="J31" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="K31" s="20" t="s">
+      <c r="K31" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L31" s="20" t="s">
+      <c r="L31" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M31" s="20">
+      <c r="M31" s="15">
         <v>35</v>
       </c>
-      <c r="N31" s="22"/>
-      <c r="O31" s="19">
+      <c r="N31" s="17"/>
+      <c r="O31" s="14">
         <v>2.66</v>
       </c>
-      <c r="P31" s="19">
+      <c r="P31" s="14">
         <f t="shared" si="0"/>
         <v>2.66</v>
       </c>
-      <c r="Q31" s="19">
+      <c r="Q31" s="14">
         <v>1.33</v>
       </c>
-      <c r="R31" s="19">
+      <c r="R31" s="14">
         <f t="shared" si="1"/>
         <v>1.33</v>
       </c>
-      <c r="S31" s="19">
+      <c r="S31" s="14">
         <f t="shared" si="2"/>
         <v>0.53200000000000003</v>
       </c>
-      <c r="T31" s="19">
+      <c r="T31" s="14">
         <f t="shared" si="3"/>
         <v>0.53200000000000003</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="14">
+      <c r="A32" s="9">
         <v>22</v>
       </c>
-      <c r="B32" s="14">
+      <c r="B32" s="9">
         <v>1</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="D32" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="F32" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="G32" s="40"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="20" t="s">
+      <c r="G32" s="35"/>
+      <c r="H32" s="35"/>
+      <c r="I32" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="J32" s="21" t="s">
+      <c r="J32" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="K32" s="20" t="s">
+      <c r="K32" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L32" s="20" t="s">
+      <c r="L32" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M32" s="20">
+      <c r="M32" s="15">
         <v>6</v>
       </c>
-      <c r="N32" s="22"/>
-      <c r="O32" s="19">
+      <c r="N32" s="17"/>
+      <c r="O32" s="14">
         <v>4.5599999999999996</v>
       </c>
-      <c r="P32" s="19">
+      <c r="P32" s="14">
         <f t="shared" si="0"/>
         <v>4.5599999999999996</v>
       </c>
-      <c r="Q32" s="19">
+      <c r="Q32" s="14">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R32" s="19">
+      <c r="R32" s="14">
         <f t="shared" si="1"/>
         <v>2.2999999999999998</v>
       </c>
-      <c r="S32" s="19">
+      <c r="S32" s="14">
         <f t="shared" si="2"/>
         <v>0.91999999999999993</v>
       </c>
-      <c r="T32" s="19">
+      <c r="T32" s="14">
         <f t="shared" si="3"/>
         <v>0.91999999999999993</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="14">
+      <c r="A33" s="9">
         <v>23</v>
       </c>
-      <c r="B33" s="14">
+      <c r="B33" s="9">
         <v>2</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="D33" s="14" t="s">
+      <c r="D33" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="E33" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F33" s="14" t="s">
+      <c r="F33" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="20" t="s">
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J33" s="21" t="s">
+      <c r="J33" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="K33" s="20" t="s">
+      <c r="K33" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L33" s="20" t="s">
+      <c r="L33" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M33" s="20">
+      <c r="M33" s="15">
         <v>14</v>
       </c>
-      <c r="N33" s="22"/>
-      <c r="O33" s="19">
+      <c r="N33" s="17"/>
+      <c r="O33" s="14">
         <v>4</v>
       </c>
-      <c r="P33" s="19">
+      <c r="P33" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="Q33" s="19">
+      <c r="Q33" s="14">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R33" s="19">
+      <c r="R33" s="14">
         <f t="shared" si="1"/>
         <v>4.5999999999999996</v>
       </c>
-      <c r="S33" s="19">
+      <c r="S33" s="14">
         <f t="shared" si="2"/>
         <v>0.91999999999999993</v>
       </c>
-      <c r="T33" s="19">
+      <c r="T33" s="14">
         <f t="shared" si="3"/>
         <v>1.8399999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="14">
+      <c r="A34" s="9">
         <v>24</v>
       </c>
-      <c r="B34" s="14">
+      <c r="B34" s="9">
         <v>3</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="C34" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="F34" s="14" t="s">
+      <c r="F34" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="20" t="s">
+      <c r="G34" s="35"/>
+      <c r="H34" s="35"/>
+      <c r="I34" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J34" s="21" t="s">
+      <c r="J34" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="K34" s="20" t="s">
+      <c r="K34" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L34" s="20" t="s">
+      <c r="L34" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M34" s="20">
+      <c r="M34" s="15">
         <v>26</v>
       </c>
-      <c r="N34" s="25"/>
-      <c r="O34" s="19">
+      <c r="N34" s="20"/>
+      <c r="O34" s="14">
         <v>2.9</v>
       </c>
-      <c r="P34" s="19">
+      <c r="P34" s="14">
         <f t="shared" si="0"/>
         <v>8.6999999999999993</v>
       </c>
-      <c r="Q34" s="19">
+      <c r="Q34" s="14">
         <v>1.7</v>
       </c>
-      <c r="R34" s="19">
+      <c r="R34" s="14">
         <f t="shared" si="1"/>
         <v>5.0999999999999996</v>
       </c>
-      <c r="S34" s="19">
+      <c r="S34" s="14">
         <f t="shared" si="2"/>
         <v>0.68</v>
       </c>
-      <c r="T34" s="19">
+      <c r="T34" s="14">
         <f t="shared" si="3"/>
         <v>2.04</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="14">
+      <c r="A35" s="9">
         <v>25</v>
       </c>
-      <c r="B35" s="14">
+      <c r="B35" s="9">
         <v>5</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="C35" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="F35" s="14" t="s">
+      <c r="F35" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="G35" s="40"/>
-      <c r="H35" s="40"/>
-      <c r="I35" s="20" t="s">
+      <c r="G35" s="35"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="J35" s="21" t="s">
+      <c r="J35" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="K35" s="20" t="s">
+      <c r="K35" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="L35" s="20" t="s">
+      <c r="L35" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M35" s="20">
+      <c r="M35" s="15">
         <v>43</v>
       </c>
-      <c r="N35" s="25"/>
-      <c r="O35" s="19">
+      <c r="N35" s="20"/>
+      <c r="O35" s="14">
         <v>0.14000000000000001</v>
       </c>
-      <c r="P35" s="19">
+      <c r="P35" s="14">
         <f t="shared" si="0"/>
         <v>0.70000000000000007</v>
       </c>
-      <c r="Q35" s="19">
+      <c r="Q35" s="14">
         <v>0.02</v>
       </c>
-      <c r="R35" s="19">
+      <c r="R35" s="14">
         <f>Q35*B35</f>
         <v>0.1</v>
       </c>
-      <c r="S35" s="19">
+      <c r="S35" s="14">
         <f>Q35*0.4</f>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="T35" s="19">
+      <c r="T35" s="14">
         <f t="shared" si="3"/>
         <v>0.04</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="31" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="26">
+    <row r="36" spans="1:20" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="21">
         <v>26</v>
       </c>
-      <c r="B36" s="26">
+      <c r="B36" s="21">
         <v>2</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="D36" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="F36" s="26" t="s">
+      <c r="F36" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="41"/>
-      <c r="H36" s="41"/>
-      <c r="I36" s="27" t="s">
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="J36" s="28" t="s">
+      <c r="J36" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="K36" s="29" t="s">
+      <c r="K36" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="L36" s="28" t="s">
+      <c r="L36" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="M36" s="28">
+      <c r="M36" s="23">
         <v>26</v>
       </c>
-      <c r="N36" s="28"/>
-      <c r="O36" s="30"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="30"/>
-      <c r="R36" s="30"/>
-      <c r="S36" s="30"/>
-      <c r="T36" s="30"/>
+      <c r="N36" s="23"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="25"/>
+      <c r="Q36" s="25"/>
+      <c r="R36" s="25"/>
+      <c r="S36" s="25"/>
+      <c r="T36" s="25"/>
     </row>
-    <row r="37" spans="1:20" s="31" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="26">
+    <row r="37" spans="1:20" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="21">
         <v>27</v>
       </c>
-      <c r="B37" s="26">
+      <c r="B37" s="21">
         <v>2</v>
       </c>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="D37" s="32" t="s">
+      <c r="D37" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E37" s="32" t="s">
+      <c r="E37" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="F37" s="32" t="s">
+      <c r="F37" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G37" s="42"/>
-      <c r="H37" s="42"/>
-      <c r="I37" s="33" t="s">
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+      <c r="I37" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="J37" s="34">
+      <c r="J37" s="29">
         <v>603</v>
       </c>
-      <c r="K37" s="33" t="s">
+      <c r="K37" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="L37" s="28" t="s">
+      <c r="L37" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="M37" s="28">
+      <c r="M37" s="23">
         <v>20</v>
       </c>
-      <c r="N37" s="28"/>
-      <c r="O37" s="30"/>
-      <c r="P37" s="30"/>
-      <c r="Q37" s="30"/>
-      <c r="R37" s="30"/>
-      <c r="S37" s="30"/>
-      <c r="T37" s="30"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="Q37" s="25"/>
+      <c r="R37" s="25"/>
+      <c r="S37" s="25"/>
+      <c r="T37" s="25"/>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="O38" s="35"/>
-      <c r="P38" s="35"/>
-      <c r="Q38" s="35"/>
-      <c r="R38" s="35"/>
-      <c r="S38" s="35"/>
-      <c r="T38" s="35"/>
+      <c r="O38" s="30"/>
+      <c r="P38" s="30"/>
+      <c r="Q38" s="30"/>
+      <c r="R38" s="30"/>
+      <c r="S38" s="30"/>
+      <c r="T38" s="30"/>
     </row>
     <row r="39" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="36" t="s">
+      <c r="A39" s="31" t="s">
         <v>156</v>
       </c>
-      <c r="O39" s="19" t="s">
+      <c r="O39" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="P39" s="19">
+      <c r="P39" s="14">
         <f>SUM(P11:P38)</f>
         <v>56.67</v>
       </c>
-      <c r="Q39" s="19"/>
-      <c r="R39" s="19">
+      <c r="Q39" s="14"/>
+      <c r="R39" s="14">
         <f>SUM(R11:R38)</f>
         <v>25.923999999999999</v>
       </c>
-      <c r="S39" s="19"/>
-      <c r="T39" s="19">
+      <c r="S39" s="14"/>
+      <c r="T39" s="14">
         <f>SUM(T11:T38)</f>
         <v>10.369599999999998</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="37" t="s">
+      <c r="A40" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="19"/>
+      <c r="O40" s="14"/>
+      <c r="P40" s="14"/>
+      <c r="Q40" s="14"/>
+      <c r="R40" s="14"/>
+      <c r="S40" s="14"/>
+      <c r="T40" s="14"/>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A41" s="38" t="s">
+      <c r="A41" s="33" t="s">
         <v>159</v>
       </c>
       <c r="D41"/>
       <c r="E41" t="s">
         <v>160</v>
       </c>
-      <c r="F41" s="38" t="s">
+      <c r="F41" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
       <c r="I41"/>
     </row>
     <row r="54" spans="1:1026" x14ac:dyDescent="0.25">
-      <c r="A54" s="39" t="s">
+      <c r="A54" s="34" t="s">
         <v>162</v>
       </c>
       <c r="B54"/>
@@ -4286,126 +4296,126 @@
       <c r="AML54"/>
     </row>
     <row r="55" spans="1:1026" x14ac:dyDescent="0.25">
-      <c r="A55" s="37" t="s">
+      <c r="A55" s="32" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="56" spans="1:1026" s="31" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="26">
+    <row r="56" spans="1:1026" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A56" s="21">
         <v>26</v>
       </c>
-      <c r="B56" s="26">
+      <c r="B56" s="21">
         <v>2</v>
       </c>
-      <c r="C56" s="26" t="s">
+      <c r="C56" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="D56" s="26" t="s">
+      <c r="D56" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="E56" s="26" t="s">
+      <c r="E56" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="F56" s="26" t="s">
+      <c r="F56" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="G56" s="26"/>
-      <c r="H56" s="26"/>
-      <c r="I56" s="26" t="s">
+      <c r="G56" s="21"/>
+      <c r="H56" s="21"/>
+      <c r="I56" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="J56" s="28" t="s">
+      <c r="J56" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="K56" s="34" t="s">
+      <c r="K56" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="L56" s="28" t="s">
+      <c r="L56" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="M56" s="28">
+      <c r="M56" s="23">
         <v>26</v>
       </c>
-      <c r="N56" s="28"/>
-      <c r="O56" s="30">
+      <c r="N56" s="23"/>
+      <c r="O56" s="25">
         <v>0.14000000000000001</v>
       </c>
-      <c r="P56" s="30">
+      <c r="P56" s="25">
         <f>B56*O56</f>
         <v>0.28000000000000003</v>
       </c>
-      <c r="Q56" s="30">
+      <c r="Q56" s="25">
         <v>2.862E-2</v>
       </c>
-      <c r="R56" s="30">
+      <c r="R56" s="25">
         <f>Q56*B56</f>
         <v>5.7239999999999999E-2</v>
       </c>
-      <c r="S56" s="30">
+      <c r="S56" s="25">
         <f>Q56*0.4</f>
         <v>1.1448E-2</v>
       </c>
-      <c r="T56" s="30">
+      <c r="T56" s="25">
         <f>B56*S56</f>
         <v>2.2896E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:1026" s="31" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="26">
+    <row r="57" spans="1:1026" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="21">
         <v>27</v>
       </c>
-      <c r="B57" s="26">
+      <c r="B57" s="21">
         <v>2</v>
       </c>
-      <c r="C57" s="26" t="s">
+      <c r="C57" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="D57" s="26" t="s">
+      <c r="D57" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="E57" s="26" t="s">
+      <c r="E57" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="F57" s="26" t="s">
+      <c r="F57" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="G57" s="26"/>
-      <c r="H57" s="26"/>
-      <c r="I57" s="28" t="s">
+      <c r="G57" s="21"/>
+      <c r="H57" s="21"/>
+      <c r="I57" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="J57" s="34">
+      <c r="J57" s="29">
         <v>603</v>
       </c>
-      <c r="K57" s="28" t="s">
+      <c r="K57" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="L57" s="28" t="s">
+      <c r="L57" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="M57" s="28">
+      <c r="M57" s="23">
         <v>20</v>
       </c>
-      <c r="N57" s="28"/>
-      <c r="O57" s="30">
+      <c r="N57" s="23"/>
+      <c r="O57" s="25">
         <v>0.1</v>
       </c>
-      <c r="P57" s="30">
+      <c r="P57" s="25">
         <f>B57*O57</f>
         <v>0.2</v>
       </c>
-      <c r="Q57" s="30">
+      <c r="Q57" s="25">
         <v>3.7799999999999999E-3</v>
       </c>
-      <c r="R57" s="30">
+      <c r="R57" s="25">
         <f>Q57*B57</f>
         <v>7.5599999999999999E-3</v>
       </c>
-      <c r="S57" s="30">
+      <c r="S57" s="25">
         <f>Q57*0.4</f>
         <v>1.5120000000000001E-3</v>
       </c>
-      <c r="T57" s="30">
+      <c r="T57" s="25">
         <f>B57*S57</f>
         <v>3.0240000000000002E-3</v>
       </c>

</xml_diff>